<commit_message>
Guía de pruebas en Excel y hoja «Pruebas» en el libro de demostración
Paso a paso con un código por prueba y su resultado esperado, medido con
el motor. La hoja nueva cubre funciones RIESGO, LET, matrices, derrame,
entradas con fórmula en el modo compatible y datos para el ajuste.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DWhE6heHjr98KiS7RpqZfr
</commit_message>
<xml_diff>
--- a/ejemplos/demo-proyecto-aurora.xlsx
+++ b/ejemplos/demo-proyecto-aurora.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Modelo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Pruebas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,9 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0 €"/>
     <numFmt numFmtId="165" formatCode="0,0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -53,7 +55,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +65,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -99,6 +106,9 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1537,4 +1547,398 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:K44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Hoja de pruebas — funciones nuevas</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Las celdas en amarillo claro están vacías a propósito: escribe en ellas la fórmula que indica la guía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>1. FUNCIONES RIESGO (prueba E)</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>5. PRECIOS HISTÓRICOS (prueba D)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Demanda — escribe =RIESGO.NORMAL(1000;150)</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="n"/>
+      <c r="K5" s="16" t="n">
+        <v>134.47</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Precio — escribe =RIESGO.TRIANGULAR(8;10;14)</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="n"/>
+      <c r="K6" s="16" t="n">
+        <v>122.61</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ingresos = Demanda × Precio</t>
+        </is>
+      </c>
+      <c r="C7" s="16">
+        <f>C5*C6</f>
+        <v/>
+      </c>
+      <c r="K7" s="16" t="n">
+        <v>165.8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="K8" s="16" t="n">
+        <v>109.42</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2. LET (prueba F)</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="n">
+        <v>119.27</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Margen = ingresos − coste (60 %), con LET</t>
+        </is>
+      </c>
+      <c r="C10" s="16">
+        <f>_xlfn.LET(_xlpm.coste,C7*0.6,C7-_xlpm.coste)</f>
+        <v/>
+      </c>
+      <c r="K10" s="16" t="n">
+        <v>125.32</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="K11" s="16" t="n">
+        <v>124.26</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>3. MATRICES (prueba G) — umbral de ventas:</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>100</v>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Derrame — escribe en H13: =FILTRAR(E13:E17;F13:F17&gt;C12)</t>
+        </is>
+      </c>
+      <c r="K12" s="16" t="n">
+        <v>119.52</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Ventas por encima del umbral — =SUMA(FILTRAR(F13:F17;F13:F17&gt;C12;0))</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="n"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="F13" s="17">
+        <f>120*$C$5/1000</f>
+        <v/>
+      </c>
+      <c r="H13" s="15" t="n"/>
+      <c r="K13" s="16" t="n">
+        <v>140.21</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Lo mismo — =SUMAPRODUCTO((F13:F17&gt;C12)*F13:F17)</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="n"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Sur</t>
+        </is>
+      </c>
+      <c r="F14" s="17">
+        <f>80*$C$5/1000</f>
+        <v/>
+      </c>
+      <c r="K14" s="16" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>La mayor — =INDICE(ORDENAR(F13:F17;1;-1);1)</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="n"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Este</t>
+        </is>
+      </c>
+      <c r="F15" s="17">
+        <f>150*$C$5/1000</f>
+        <v/>
+      </c>
+      <c r="K15" s="16" t="n">
+        <v>119.96</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Oeste</t>
+        </is>
+      </c>
+      <c r="F16" s="17">
+        <f>60*$C$5/1000</f>
+        <v/>
+      </c>
+      <c r="K16" s="16" t="n">
+        <v>118.43</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Centro</t>
+        </is>
+      </c>
+      <c r="F17" s="17">
+        <f>200*$C$5/1000</f>
+        <v/>
+      </c>
+      <c r="K17" s="16" t="n">
+        <v>123.06</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="K18" s="16" t="n">
+        <v>103.96</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="K19" s="16" t="n">
+        <v>123.39</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>4. ENTRADA CON FÓRMULA (prueba H)</t>
+        </is>
+      </c>
+      <c r="K20" s="16" t="n">
+        <v>114.93</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Coste unitario (es una fórmula: =7+1)</t>
+        </is>
+      </c>
+      <c r="C21">
+        <f>7+1</f>
+        <v/>
+      </c>
+      <c r="K21" s="16" t="n">
+        <v>120.58</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Coste total = coste unitario × demanda</t>
+        </is>
+      </c>
+      <c r="C22" s="16">
+        <f>C21*C5</f>
+        <v/>
+      </c>
+      <c r="K22" s="16" t="n">
+        <v>123.19</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="K23" s="16" t="n">
+        <v>122.39</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="K24" s="16" t="n">
+        <v>135.13</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="K25" s="16" t="n">
+        <v>107.99</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="K26" s="16" t="n">
+        <v>128.92</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="K27" s="16" t="n">
+        <v>117.6</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="K28" s="16" t="n">
+        <v>114.05</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="K29" s="16" t="n">
+        <v>104.62</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="K30" s="16" t="n">
+        <v>102.97</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="K31" s="16" t="n">
+        <v>114.72</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="K32" s="16" t="n">
+        <v>92.87</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="K33" s="16" t="n">
+        <v>90.79000000000001</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="K34" s="16" t="n">
+        <v>105.47</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="K35" s="16" t="n">
+        <v>115.54</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="K36" s="16" t="n">
+        <v>105.38</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="K37" s="16" t="n">
+        <v>138.82</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="K38" s="16" t="n">
+        <v>131.28</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="K39" s="16" t="n">
+        <v>95.36</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="K40" s="16" t="n">
+        <v>120.34</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="K41" s="16" t="n">
+        <v>131.99</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="K42" s="16" t="n">
+        <v>108.7</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="K43" s="16" t="n">
+        <v>113.68</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="K44" s="16" t="n">
+        <v>121.08</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Guía de pruebas reescrita desde cero y libro de demostración con la hoja Zonas
La guía recorre todo el complemento de principio a fin (0, A–H, T, J, K, W, I),
incluidas la etapa 1b, las variables de texto y lo hecho antes de la etapa 2.
El libro de demostración añade la hoja «Zonas» y la sección 6 de «Pruebas» con
celdas para DISCRETA, TRUNCAR, LOGNORMAL2 y EMPIRICA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DWhE6heHjr98KiS7RpqZfr
</commit_message>
<xml_diff>
--- a/ejemplos/demo-proyecto-aurora.xlsx
+++ b/ejemplos/demo-proyecto-aurora.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Modelo" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Pruebas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Zonas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -88,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -109,6 +110,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1559,8 +1562,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="8" max="8"/>
@@ -1584,22 +1588,27 @@
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1. FUNCIONES RIESGO (prueba E)</t>
+          <t>1. FUNCIONES RIESGO (pruebas F1–F6)</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>5. PRECIOS HISTÓRICOS (prueba D)</t>
+          <t>5. PRECIOS HISTÓRICOS (prueba E)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>Demanda — escribe =RIESGO.NORMAL(1000;150)</t>
+          <t>Demanda</t>
         </is>
       </c>
       <c r="C5" s="15" t="n"/>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.NORMAL(1000;150)</t>
+        </is>
+      </c>
       <c r="K5" s="16" t="n">
         <v>134.47</v>
       </c>
@@ -1607,10 +1616,15 @@
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>Precio — escribe =RIESGO.TRIANGULAR(8;10;14)</t>
+          <t>Precio</t>
         </is>
       </c>
       <c r="C6" s="15" t="n"/>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.TRIANGULAR(8;10;14)</t>
+        </is>
+      </c>
       <c r="K6" s="16" t="n">
         <v>122.61</v>
       </c>
@@ -1637,7 +1651,7 @@
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2. LET (prueba F)</t>
+          <t>2. LET (prueba G1)</t>
         </is>
       </c>
       <c r="K9" s="16" t="n">
@@ -1659,6 +1673,11 @@
       </c>
     </row>
     <row r="11">
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>Derrame — escribe en H13: =FILTRAR(E13:E17;F13:F17&gt;C12)</t>
+        </is>
+      </c>
       <c r="K11" s="16" t="n">
         <v>124.26</v>
       </c>
@@ -1666,7 +1685,7 @@
     <row r="12">
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>3. MATRICES (prueba G) — umbral de ventas:</t>
+          <t>3. MATRICES (pruebas G2–G4) — umbral de ventas:</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1682,11 +1701,6 @@
           <t>Ventas</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>Derrame — escribe en H13: =FILTRAR(E13:E17;F13:F17&gt;C12)</t>
-        </is>
-      </c>
       <c r="K12" s="16" t="n">
         <v>119.52</v>
       </c>
@@ -1694,7 +1708,7 @@
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ventas por encima del umbral — =SUMA(FILTRAR(F13:F17;F13:F17&gt;C12;0))</t>
+          <t>Ventas por encima del umbral</t>
         </is>
       </c>
       <c r="C13" s="15" t="n"/>
@@ -1708,6 +1722,11 @@
         <v/>
       </c>
       <c r="H13" s="15" t="n"/>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>escribe =SUMA(FILTRAR(F13:F17;F13:F17&gt;C12;0))</t>
+        </is>
+      </c>
       <c r="K13" s="16" t="n">
         <v>140.21</v>
       </c>
@@ -1715,7 +1734,7 @@
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>Lo mismo — =SUMAPRODUCTO((F13:F17&gt;C12)*F13:F17)</t>
+          <t>Ventas por encima del umbral (SUMAPRODUCTO)</t>
         </is>
       </c>
       <c r="C14" s="15" t="n"/>
@@ -1728,6 +1747,11 @@
         <f>80*$C$5/1000</f>
         <v/>
       </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>escribe =SUMAPRODUCTO((F13:F17&gt;C12)*F13:F17)</t>
+        </is>
+      </c>
       <c r="K14" s="16" t="n">
         <v>130</v>
       </c>
@@ -1735,7 +1759,7 @@
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>La mayor — =INDICE(ORDENAR(F13:F17;1;-1);1)</t>
+          <t>La mayor venta</t>
         </is>
       </c>
       <c r="C15" s="15" t="n"/>
@@ -1747,6 +1771,11 @@
       <c r="F15" s="17">
         <f>150*$C$5/1000</f>
         <v/>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>escribe =INDICE(ORDENAR(F13:F17;1;-1);1)</t>
+        </is>
       </c>
       <c r="K15" s="16" t="n">
         <v>119.96</v>
@@ -1834,31 +1863,117 @@
       </c>
     </row>
     <row r="24">
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>6. FUNCIONES NUEVAS (pruebas F7–F10)</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Plazo</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Peso</t>
+        </is>
+      </c>
       <c r="K24" s="16" t="n">
         <v>135.13</v>
       </c>
     </row>
     <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Plazo de entrega (días)</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="n"/>
+      <c r="E25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.DISCRETA(E25:E27;F25:F27)</t>
+        </is>
+      </c>
       <c r="K25" s="16" t="n">
         <v>107.99</v>
       </c>
     </row>
     <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Demanda acotada</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="n"/>
+      <c r="E26" t="n">
+        <v>5</v>
+      </c>
+      <c r="F26" s="18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.TRUNCAR(RIESGO.NORMAL(100;30);50;150)</t>
+        </is>
+      </c>
       <c r="K26" s="16" t="n">
         <v>128.92</v>
       </c>
     </row>
     <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Precio lognormal</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="n"/>
+      <c r="E27" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.LOGNORMAL2(4,6;0,2)</t>
+        </is>
+      </c>
       <c r="K27" s="16" t="n">
         <v>117.6</v>
       </c>
     </row>
     <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Precio según el histórico</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="n"/>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.EMPIRICA(K5:K44)</t>
+        </is>
+      </c>
       <c r="K28" s="16" t="n">
         <v>114.05</v>
       </c>
     </row>
     <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Suma de control</t>
+        </is>
+      </c>
+      <c r="C29" s="16">
+        <f>C25+C26+C27+C28</f>
+        <v/>
+      </c>
       <c r="K29" s="16" t="n">
         <v>104.62</v>
       </c>
@@ -1936,6 +2051,226 @@
     <row r="44">
       <c r="K44" s="16" t="n">
         <v>121.08</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Variables de texto — zona de venta</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>La zona es un texto con su probabilidad. El recargo depende de la zona; la gama y el «¿supera?» son salidas de texto y de sí/no.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Zona de venta</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Probabilidad</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Recargo</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>marca como entrada: el panel la propone como texto</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Recargo por zona</t>
+        </is>
+      </c>
+      <c r="C5" s="19">
+        <f>VLOOKUP(C4,$E$5:$G$7,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Precio base</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Sur</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>marca como entrada</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Unidades</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Este</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>marca como entrada</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="C8" s="11">
+        <f>C6*C5*C7</f>
+        <v/>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>salida numérica</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Gama</t>
+        </is>
+      </c>
+      <c r="C9">
+        <f>IF(C8&gt;110000,"Alta",IF(C8&gt;90000,"Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>salida de texto</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>¿Supera 100.000 €?</t>
+        </is>
+      </c>
+      <c r="C10">
+        <f>C8&gt;100000</f>
+        <v/>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>salida de sí/no</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Zona con función</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="n"/>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.CATEGORIA(E5:E7;F5:F7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Ingresos con la zona de la función</t>
+        </is>
+      </c>
+      <c r="C13" s="11">
+        <f>C6*VLOOKUP(C12,$E$5:$G$7,3,FALSE)*C7</f>
+        <v/>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>salida</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Guía, libro de demostración y documentos para B7 y B6
Secciones 7 (RIESGO con celdas) y 8 (resultados en la hoja) en la hoja
Pruebas, con sus cifras comprobadas por el motor en hojaPruebasDemo.test.ts.
Guía: F5 cambiada, pruebas F12–F19, T8 y W7, y notas en la preparación y en J.
CHANGELOG, estado, plan e inventario al día.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DWhE6heHjr98KiS7RpqZfr
</commit_message>
<xml_diff>
--- a/ejemplos/demo-proyecto-aurora.xlsx
+++ b/ejemplos/demo-proyecto-aurora.xlsx
@@ -19,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0 €"/>
     <numFmt numFmtId="165" formatCode="0,0%"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -89,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -111,6 +112,8 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1568,6 +1571,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -1984,36 +1988,99 @@
       </c>
     </row>
     <row r="31">
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>7. RIESGO CON CELDAS (pruebas F12–F15)</t>
+        </is>
+      </c>
       <c r="K31" s="16" t="n">
         <v>114.72</v>
       </c>
     </row>
     <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Media de la demanda</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1000</v>
+      </c>
       <c r="K32" s="16" t="n">
         <v>92.87</v>
       </c>
     </row>
     <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Desviación de la demanda</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>150</v>
+      </c>
       <c r="K33" s="16" t="n">
         <v>90.79000000000001</v>
       </c>
     </row>
     <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Demanda con celdas</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="n"/>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.NORMAL(C32;C33)</t>
+        </is>
+      </c>
       <c r="K34" s="16" t="n">
         <v>105.47</v>
       </c>
     </row>
     <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Precio con imprevisto</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="n"/>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>escribe =10+RIESGO.NORMAL(0;1)</t>
+        </is>
+      </c>
       <c r="K35" s="16" t="n">
         <v>115.54</v>
       </c>
     </row>
     <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Demanda del mes siguiente</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="n"/>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.NORMAL(C34;50)</t>
+        </is>
+      </c>
       <c r="K36" s="16" t="n">
         <v>105.38</v>
       </c>
     </row>
     <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Ingresos con celdas</t>
+        </is>
+      </c>
+      <c r="C37" s="16">
+        <f>C36*C35</f>
+        <v/>
+      </c>
       <c r="K37" s="16" t="n">
         <v>138.82</v>
       </c>
@@ -2024,26 +2091,75 @@
       </c>
     </row>
     <row r="39">
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>8. RESULTADOS EN LA HOJA (pruebas F16–F19)</t>
+        </is>
+      </c>
       <c r="K39" s="16" t="n">
         <v>95.36</v>
       </c>
     </row>
     <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Media de los ingresos</t>
+        </is>
+      </c>
+      <c r="C40" s="19" t="n"/>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.MEDIA(C37)</t>
+        </is>
+      </c>
       <c r="K40" s="16" t="n">
         <v>120.34</v>
       </c>
     </row>
     <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>p5 de los ingresos</t>
+        </is>
+      </c>
+      <c r="C41" s="19" t="n"/>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.PERCENTIL(C37;0,05)</t>
+        </is>
+      </c>
       <c r="K41" s="16" t="n">
         <v>131.99</v>
       </c>
     </row>
     <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Probabilidad de ingresos &lt; 8.000</t>
+        </is>
+      </c>
+      <c r="C42" s="20" t="n"/>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.PROB(C37;8000)</t>
+        </is>
+      </c>
       <c r="K42" s="16" t="n">
         <v>108.7</v>
       </c>
     </row>
     <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Desviación de los ingresos</t>
+        </is>
+      </c>
+      <c r="C43" s="19" t="n"/>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.DESV(C37)</t>
+        </is>
+      </c>
       <c r="K43" s="16" t="n">
         <v>113.68</v>
       </c>
@@ -2128,7 +2244,7 @@
           <t>Recargo por zona</t>
         </is>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="21">
         <f>VLOOKUP(C4,$E$5:$G$7,3,FALSE)</f>
         <v/>
       </c>
@@ -2140,7 +2256,7 @@
       <c r="F5" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="19" t="n">
+      <c r="G5" s="21" t="n">
         <v>1.1</v>
       </c>
     </row>
@@ -2161,7 +2277,7 @@
       <c r="F6" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="G6" s="19" t="n">
+      <c r="G6" s="21" t="n">
         <v>1</v>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -2187,7 +2303,7 @@
       <c r="F7" s="18" t="n">
         <v>0.3</v>
       </c>
-      <c r="G7" s="19" t="n">
+      <c r="G7" s="21" t="n">
         <v>0.9</v>
       </c>
       <c r="I7" s="4" t="inlineStr">

</xml_diff>

<commit_message>
B6: RIESGO.SALIDA y RIESGO.CORRELACION
Marcar salidas y correlacionar entradas desde la fórmula; Simular ya no
exige salidas en el panel. Compartir deja la salida calculando y lleva al
panel lo declarado. Banco con formulas= y valores que quitan la fórmula.
Demo sección 9, guía F20, F21 y N12.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DWhE6heHjr98KiS7RpqZfr
</commit_message>
<xml_diff>
--- a/ejemplos/demo-proyecto-aurora.xlsx
+++ b/ejemplos/demo-proyecto-aurora.xlsx
@@ -90,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -114,6 +114,7 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1561,7 +1562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:K44"/>
+  <dimension ref="B2:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2167,6 +2168,65 @@
     <row r="44">
       <c r="K44" s="16" t="n">
         <v>121.08</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>9. SALIDA Y CORRELACIÓN CON FUNCIONES (pruebas F20–F21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Coste de materiales</t>
+        </is>
+      </c>
+      <c r="C46" s="19" t="n"/>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.NORMAL(100;10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Coste de transporte</t>
+        </is>
+      </c>
+      <c r="C47" s="19" t="n"/>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.NORMAL(50;5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Correlación materiales-transporte</t>
+        </is>
+      </c>
+      <c r="C48" s="21" t="n"/>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.CORRELACION(C46;C47;0,9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Coste total</t>
+        </is>
+      </c>
+      <c r="C49" s="19" t="n"/>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.SALIDA("Coste total")+C46+C47</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2244,7 +2304,7 @@
           <t>Recargo por zona</t>
         </is>
       </c>
-      <c r="C5" s="21">
+      <c r="C5" s="22">
         <f>VLOOKUP(C4,$E$5:$G$7,3,FALSE)</f>
         <v/>
       </c>
@@ -2256,7 +2316,7 @@
       <c r="F5" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="21" t="n">
+      <c r="G5" s="22" t="n">
         <v>1.1</v>
       </c>
     </row>
@@ -2277,7 +2337,7 @@
       <c r="F6" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="G6" s="21" t="n">
+      <c r="G6" s="22" t="n">
         <v>1</v>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -2303,7 +2363,7 @@
       <c r="F7" s="18" t="n">
         <v>0.3</v>
       </c>
-      <c r="G7" s="21" t="n">
+      <c r="G7" s="22" t="n">
         <v>0.9</v>
       </c>
       <c r="I7" s="4" t="inlineStr">

</xml_diff>

<commit_message>
T7: entradas y salidas de fecha
Las celdas con formato de fecha se enseñan como fechas en Resultados, el
informe y la hoja volcada, con la dispersión en días; la probabilidad y los
delimitadores aceptan fechas escritas. Demo sección 10, guía T9 y N14.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DWhE6heHjr98KiS7RpqZfr
</commit_message>
<xml_diff>
--- a/ejemplos/demo-proyecto-aurora.xlsx
+++ b/ejemplos/demo-proyecto-aurora.xlsx
@@ -19,11 +19,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="#,##0 €"/>
     <numFmt numFmtId="165" formatCode="0,0%"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -90,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,6 +116,9 @@
     <xf numFmtId="4" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1562,7 +1566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:K49"/>
+  <dimension ref="B2:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2227,6 +2231,50 @@
         <is>
           <t>escribe =RIESGO.SALIDA("Coste total")+C46+C47</t>
         </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>10. FECHAS (prueba T9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Inicio de obra</t>
+        </is>
+      </c>
+      <c r="C52" s="22" t="n"/>
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.TRIANGULAR(FECHA(2027;1;1);FECHA(2027;2;1);FECHA(2027;4;1))</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Duración (días)</t>
+        </is>
+      </c>
+      <c r="C53" s="23" t="n"/>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.NORMAL(90;10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Fin de obra</t>
+        </is>
+      </c>
+      <c r="C54" s="24">
+        <f>C52+C53</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -2304,7 +2352,7 @@
           <t>Recargo por zona</t>
         </is>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="25">
         <f>VLOOKUP(C4,$E$5:$G$7,3,FALSE)</f>
         <v/>
       </c>
@@ -2316,7 +2364,7 @@
       <c r="F5" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="22" t="n">
+      <c r="G5" s="25" t="n">
         <v>1.1</v>
       </c>
     </row>
@@ -2337,7 +2385,7 @@
       <c r="F6" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="G6" s="22" t="n">
+      <c r="G6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -2363,7 +2411,7 @@
       <c r="F7" s="18" t="n">
         <v>0.3</v>
       </c>
-      <c r="G7" s="22" t="n">
+      <c r="G7" s="25" t="n">
         <v>0.9</v>
       </c>
       <c r="I7" s="4" t="inlineStr">

</xml_diff>

<commit_message>
T8: registro de riesgos
RIESGO.EVENTO(probabilidad; impacto) y la sección «Registro de riesgos» en
Resultados con el valor esperado de cada riesgo y su parte del total.
Demo sección 11, guía T10 y N15.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DWhE6heHjr98KiS7RpqZfr
</commit_message>
<xml_diff>
--- a/ejemplos/demo-proyecto-aurora.xlsx
+++ b/ejemplos/demo-proyecto-aurora.xlsx
@@ -91,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,6 +119,7 @@
     <xf numFmtId="168" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1566,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:K54"/>
+  <dimension ref="B2:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2274,6 +2275,50 @@
       </c>
       <c r="C54" s="24">
         <f>C52+C53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>11. REGISTRO DE RIESGOS (prueba T10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Retraso de permisos</t>
+        </is>
+      </c>
+      <c r="C57" s="25" t="n"/>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.EVENTO(0,3;RIESGO.TRIANGULAR(10000;20000;60000))</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Avería grave</t>
+        </is>
+      </c>
+      <c r="C58" s="25" t="n"/>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.EVENTO(0,1;50000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Coste de los riesgos</t>
+        </is>
+      </c>
+      <c r="C59" s="10">
+        <f>C57+C58</f>
         <v/>
       </c>
     </row>
@@ -2352,7 +2397,7 @@
           <t>Recargo por zona</t>
         </is>
       </c>
-      <c r="C5" s="25">
+      <c r="C5" s="26">
         <f>VLOOKUP(C4,$E$5:$G$7,3,FALSE)</f>
         <v/>
       </c>
@@ -2364,7 +2409,7 @@
       <c r="F5" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="25" t="n">
+      <c r="G5" s="26" t="n">
         <v>1.1</v>
       </c>
     </row>
@@ -2385,7 +2430,7 @@
       <c r="F6" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="G6" s="25" t="n">
+      <c r="G6" s="26" t="n">
         <v>1</v>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -2411,7 +2456,7 @@
       <c r="F7" s="18" t="n">
         <v>0.3</v>
       </c>
-      <c r="G7" s="25" t="n">
+      <c r="G7" s="26" t="n">
         <v>0.9</v>
       </c>
       <c r="I7" s="4" t="inlineStr">

</xml_diff>

<commit_message>
T9: opciones de decisión
RIESGO.DECISION con opciones escritas o un rango; al simular, cada opción
(o combinación, hasta 16) con los mismos números aleatorios, y la tabla
«Comparar decisiones» en Resultados. Demo sección 12, guía T11 y N16.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DWhE6heHjr98KiS7RpqZfr
</commit_message>
<xml_diff>
--- a/ejemplos/demo-proyecto-aurora.xlsx
+++ b/ejemplos/demo-proyecto-aurora.xlsx
@@ -1567,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:K59"/>
+  <dimension ref="B2:K64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2319,6 +2319,50 @@
       </c>
       <c r="C59" s="10">
         <f>C57+C58</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>12. DECISIONES (prueba T11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Demanda</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="n"/>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.NORMAL(1000;100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Precio (decisión)</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="n"/>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.DECISION(8;10;12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Ingresos según el precio</t>
+        </is>
+      </c>
+      <c r="C64" s="10">
+        <f>C62*C63</f>
         <v/>
       </c>
     </row>

</xml_diff>